<commit_message>
feat: integrate PieChartWrapper component for consistent pie chart rendering across dashboards and statistics pages
</commit_message>
<xml_diff>
--- a/Backend/uploads/1747473177725.xlsx
+++ b/Backend/uploads/1747473177725.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\coding\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Election-System-V2\Backend\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2AFC3443-D8E3-4B89-A66D-E3DA02D1EFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{C01B6C75-3855-4798-9F6C-3C0DE1DB757A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>StudentIds</t>
   </si>
@@ -58,12 +57,45 @@
   </si>
   <si>
     <t>STU-2026-0010</t>
+  </si>
+  <si>
+    <t>Alain</t>
+  </si>
+  <si>
+    <t>Caleb</t>
+  </si>
+  <si>
+    <t>Nyaxo</t>
+  </si>
+  <si>
+    <t>Joe</t>
+  </si>
+  <si>
+    <t>Keza</t>
+  </si>
+  <si>
+    <t>Sati</t>
+  </si>
+  <si>
+    <t>Joshua</t>
+  </si>
+  <si>
+    <t>Jane</t>
+  </si>
+  <si>
+    <t>Camella</t>
+  </si>
+  <si>
+    <t>Job</t>
+  </si>
+  <si>
+    <t>Names</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -408,66 +440,99 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EA2DBB9-4313-4841-98F0-74F2D1F34918}">
-  <dimension ref="A1:A20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" customWidth="1"/>
+    <col min="1" max="1" width="18.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>10</v>
+      </c>
+      <c r="B20" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>